<commit_message>
Review against the submission checklist: fix report claims, add run logs
- run_logs/: config, per-epoch history and summary of all 21 runs plus the
  stage stdout logs, so every number traces to an exp_id and a log line.
- Report: 3-seed check shows CutMix has no effect (val 1-view 0.9680 vs
  0.9684) and the final gain comes from 288 px inference; ResNet-50
  underfits while EfficientNet/MobileNet show the BN train/val gap; fix the
  T10/EMA explanation to match its curve; add a training-curve section,
  embedded figures and a missed-weeds error analysis.
- results.xlsx: curve links point at the per-seed T00/F01 images.
- Re-running is safe: eda/sanity/bnrecal/inference skip when their tables
  exist (--force to recompute); notebook grades with the I04 288 latency.
- README: Colab links and run_logs.
</commit_message>
<xml_diff>
--- a/submissions/2A202602505_van_quoc_dung/results.xlsx
+++ b/submissions/2A202602505_van_quoc_dung/results.xlsx
@@ -1502,7 +1502,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>curves/T00_baseline.png</t>
+          <t>curves/T00_baseline_seed0.png</t>
         </is>
       </c>
       <c r="P2">
@@ -3450,7 +3450,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:O10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -3467,6 +3467,7 @@
     <col width="20" customWidth="1" min="12" max="12"/>
     <col width="20" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="31" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3540,6 +3541,11 @@
           <t>pred_file</t>
         </is>
       </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>curve</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3590,6 +3596,11 @@
           <t>F01_seed0_test.csv</t>
         </is>
       </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>curves/F01_final_seed0.png</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3640,6 +3651,11 @@
           <t>F01_seed1_test.csv</t>
         </is>
       </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>curves/F01_final_seed1.png</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3690,6 +3706,11 @@
           <t>F01_seed2_test.csv</t>
         </is>
       </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>curves/F01_final_seed2.png</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -3794,6 +3815,11 @@
           <t>T00_seed0_test.csv</t>
         </is>
       </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>curves/T00_baseline_seed0.png</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -3841,6 +3867,11 @@
           <t>T00_seed1_test.csv</t>
         </is>
       </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>curves/T00_baseline_seed1.png</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -3886,6 +3917,11 @@
       <c r="N8" t="inlineStr">
         <is>
           <t>T00_seed2_test.csv</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>curves/T00_baseline_seed2.png</t>
         </is>
       </c>
     </row>

</xml_diff>